<commit_message>
Testplan en experimenteel onderzoek verder ingevuld, test 1, 2, en 6, afgerond
</commit_message>
<xml_diff>
--- a/Opleverset/Extra documenten/Excel sheets/Uitgaves_Floating_Farm.xlsx
+++ b/Opleverset/Extra documenten/Excel sheets/Uitgaves_Floating_Farm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtha\Documents\GitHub\Project-5-6---Floating-Farm\Opleverset\Extra documenten\Excel sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B22B106-502C-4193-80B4-186112843703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C89596E0-24D0-45F4-A499-FD3C749E493D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="19200" windowHeight="11170" xr2:uid="{14AEBCC3-6D87-4B1A-9D64-0CD8C4A83626}"/>
+    <workbookView xWindow="1050" yWindow="1560" windowWidth="19200" windowHeight="11170" xr2:uid="{14AEBCC3-6D87-4B1A-9D64-0CD8C4A83626}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -86,7 +86,7 @@
     <t>Houten plaat, prototype 2</t>
   </si>
   <si>
-    <t>Arcylplaat 25x50cm</t>
+    <t>Arcylplaat 50x100cm</t>
   </si>
 </sst>
 </file>
@@ -500,7 +500,7 @@
       </c>
       <c r="E2" s="1">
         <f>SUM(B2:B1048576)</f>
-        <v>78.490000000000009</v>
+        <v>82.580000000000013</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -591,7 +591,7 @@
         <v>16</v>
       </c>
       <c r="B13">
-        <v>12</v>
+        <v>16.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Testplan en Uitgaves aangepast
</commit_message>
<xml_diff>
--- a/Opleverset/Extra documenten/Excel sheets/Uitgaves_Floating_Farm.xlsx
+++ b/Opleverset/Extra documenten/Excel sheets/Uitgaves_Floating_Farm.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtha\Documents\GitHub\Project-5-6---Floating-Farm\Opleverset\Extra documenten\Excel sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CFBE3CD-CF80-4B0B-AF48-526A6DFC69ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{564E44ED-DC1D-43A1-B43A-52226D6D6E7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1050" yWindow="1560" windowWidth="19200" windowHeight="11170" xr2:uid="{14AEBCC3-6D87-4B1A-9D64-0CD8C4A83626}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Item</t>
   </si>
@@ -65,18 +65,6 @@
     <t>ESP-WROOM-32 microcontroller</t>
   </si>
   <si>
-    <t>Jumper cables Pcs 40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4x BS170 Mosfet </t>
-  </si>
-  <si>
-    <t>100x  10k ohm weerstand</t>
-  </si>
-  <si>
-    <t>4x DC connector male adapters</t>
-  </si>
-  <si>
     <t>Opbergbox voor demonstratie</t>
   </si>
   <si>
@@ -87,6 +75,12 @@
   </si>
   <si>
     <t>Arcylplaat 50x100cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4x IRFZ44N Mosfet </t>
+  </si>
+  <si>
+    <t>Alle andere kosten zijn verwaarloosbaar, waaronder Kabels, weerstandjes, lampjes en tape/plakspul</t>
   </si>
 </sst>
 </file>
@@ -500,7 +494,7 @@
       </c>
       <c r="E2" s="1">
         <f>SUM(B2:B1048576)</f>
-        <v>82.580000000000013</v>
+        <v>64.180000000000007</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -519,7 +513,7 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <v>4.95</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -527,15 +521,15 @@
         <v>8</v>
       </c>
       <c r="B5">
-        <v>12.41</v>
+        <v>6.67</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B6">
-        <v>3.11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -543,55 +537,36 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>6.99</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8">
-        <v>1.49</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9">
-        <v>1.61</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10">
-        <v>3.82</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11">
-        <v>0.65</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12">
-        <v>5</v>
+        <v>16.09</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13">
-        <v>16.09</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Folders aangepast, en laatste dingen aan teamreflectie en uitgaves
</commit_message>
<xml_diff>
--- a/Opleverset/Extra documenten/Excel sheets/Uitgaves_Floating_Farm.xlsx
+++ b/Opleverset/Extra documenten/Excel sheets/Uitgaves_Floating_Farm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtha\Documents\GitHub\Project-5-6---Floating-Farm\Opleverset\Extra documenten\Excel sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{564E44ED-DC1D-43A1-B43A-52226D6D6E7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A623B1DD-9BBE-4C82-902A-F01C92011AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1050" yWindow="1560" windowWidth="19200" windowHeight="11170" xr2:uid="{14AEBCC3-6D87-4B1A-9D64-0CD8C4A83626}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Item</t>
   </si>
@@ -48,12 +48,6 @@
   </si>
   <si>
     <t>Houten plaat, prototype 1</t>
-  </si>
-  <si>
-    <t>Datum</t>
-  </si>
-  <si>
-    <t>19/09/2025</t>
   </si>
   <si>
     <t>Mini Waterpomp x4 + buizen</t>
@@ -458,7 +452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68DF2FA7-E7C3-4436-AF28-B59F61D87239}">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="37.26953125" customWidth="1"/>
@@ -468,105 +462,98 @@
     <col min="8" max="8" width="37.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="1">
         <v>5</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" s="1">
+      <c r="C2" s="3"/>
+      <c r="D2" s="1">
         <f>SUM(B2:B1048576)</f>
         <v>64.180000000000007</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B3">
         <v>21.46</v>
       </c>
-      <c r="C3" s="2">
-        <v>45758</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B4">
         <v>3.49</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B5">
         <v>6.67</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B7">
         <v>3.82</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B8">
         <v>0.65</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B9">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B10">
         <v>16.09</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feedback opdrachtgever genoteerd, uitgaves aangepast en gebruikeronderzoek verbeter (nog niet klaar)
</commit_message>
<xml_diff>
--- a/Opleverset/Extra documenten/Excel sheets/Uitgaves_Floating_Farm.xlsx
+++ b/Opleverset/Extra documenten/Excel sheets/Uitgaves_Floating_Farm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtha\Documents\GitHub\Project-5-6---Floating-Farm\Opleverset\Extra documenten\Excel sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5BBF41E-C5CE-4243-B6FE-9143FFA0E152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85FA4F51-8D26-4067-A7FA-62F616304432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{14AEBCC3-6D87-4B1A-9D64-0CD8C4A83626}"/>
+    <workbookView xWindow="1900" yWindow="1280" windowWidth="19200" windowHeight="11170" xr2:uid="{14AEBCC3-6D87-4B1A-9D64-0CD8C4A83626}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Item</t>
   </si>
@@ -75,6 +75,12 @@
   </si>
   <si>
     <t>Alle andere kosten zijn verwaarloosbaar, waaronder Kabels, weerstandjes, lampjes en tape/plakspul</t>
+  </si>
+  <si>
+    <t>Oplaadbare batterijen 4pack x2</t>
+  </si>
+  <si>
+    <t>Bison Patafix kneedgom</t>
   </si>
 </sst>
 </file>
@@ -452,7 +458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68DF2FA7-E7C3-4436-AF28-B59F61D87239}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="37.26953125" customWidth="1"/>
@@ -483,7 +489,7 @@
       <c r="C2" s="3"/>
       <c r="D2" s="1">
         <f>SUM(B2:B1048576)</f>
-        <v>64.180000000000007</v>
+        <v>79.150000000000006</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -551,8 +557,24 @@
         <v>16.09</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11">
+        <v>13.98</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>